<commit_message>
LGFU BOG changed to SBOG
</commit_message>
<xml_diff>
--- a/scripts/Caribou/habitat_classification_withNotes.xlsx
+++ b/scripts/Caribou/habitat_classification_withNotes.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="T:\git\p3t_ArcGIS_Pro_Tools\scripts\Caribou\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\T\git\p3t_ArcGIS_Pro_Tools\scripts\Caribou\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27D82BA5-B47C-4229-B17C-CCD279A30FC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4801330-46F3-4E4C-8E36-8C285BA971CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{255018A2-ECAD-4F8E-B382-677AE40584B1}"/>
+    <workbookView xWindow="4155" yWindow="0" windowWidth="17100" windowHeight="15585" activeTab="4" xr2:uid="{255018A2-ECAD-4F8E-B382-677AE40584B1}"/>
   </bookViews>
   <sheets>
     <sheet name="notes" sheetId="2" r:id="rId1"/>
     <sheet name="main" sheetId="1" r:id="rId2"/>
+    <sheet name="CM1_3 part1" sheetId="3" r:id="rId3"/>
+    <sheet name="CM1_3 part2" sheetId="4" r:id="rId4"/>
+    <sheet name="CM1_3_part3" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -54,8 +57,71 @@
 </comments>
 </file>
 
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={2962486B-8D99-4130-8A33-5C0AE0A274D5}</author>
+    <author>tc={7C908EB8-4275-4D83-8DF4-FB495EEC1BDF}</author>
+  </authors>
+  <commentList>
+    <comment ref="A3" authorId="0" shapeId="0" xr:uid="{2962486B-8D99-4130-8A33-5C0AE0A274D5}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    There is a look-up table available to map thousands of plan forest unit to provincial standard forest units. Most CM1.3 data will be mapped to PSFU then mapped to LGFU to determine caribou habitat</t>
+      </text>
+    </comment>
+    <comment ref="C3" authorId="1" shapeId="0" xr:uid="{7C908EB8-4275-4D83-8DF4-FB495EEC1BDF}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    From Larry's PIAM 2024</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={4401C003-C0F5-4F5E-B99D-BFAE1416E019}</author>
+  </authors>
+  <commentList>
+    <comment ref="A13" authorId="0" shapeId="0" xr:uid="{4401C003-C0F5-4F5E-B99D-BFAE1416E019}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    It should’ve been SBLOW/SB1, but in this context, it seems more appropriate to assign this to SPDOM/SP1</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={CEE603A1-4FDB-4D6E-91BE-F9B21160272F}</author>
+  </authors>
+  <commentList>
+    <comment ref="A12" authorId="0" shapeId="0" xr:uid="{CEE603A1-4FDB-4D6E-91BE-F9B21160272F}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    It should’ve been SBLOW/SB1, but in this context, it seems more appropriate to assign this to SPDOM/SP1</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="128">
   <si>
     <t>BFDOM</t>
   </si>
@@ -256,13 +322,196 @@
   </si>
   <si>
     <t>BWSHA</t>
+  </si>
+  <si>
+    <t>LH1/TH1</t>
+  </si>
+  <si>
+    <t>PW1/PR1/PWR</t>
+  </si>
+  <si>
+    <t>ALL</t>
+  </si>
+  <si>
+    <t>BWDOM/BW1</t>
+  </si>
+  <si>
+    <t>BWDOM</t>
+  </si>
+  <si>
+    <t>CONMX/SF1</t>
+  </si>
+  <si>
+    <t>CONMX2/MW1</t>
+  </si>
+  <si>
+    <t>HDSEL</t>
+  </si>
+  <si>
+    <t>OTHER</t>
+  </si>
+  <si>
+    <t>HDUS</t>
+  </si>
+  <si>
+    <t>HE1</t>
+  </si>
+  <si>
+    <t>HRDDOM/MW2</t>
+  </si>
+  <si>
+    <t>OCLOW/LC1</t>
+  </si>
+  <si>
+    <t>OTH</t>
+  </si>
+  <si>
+    <t>OTHHD/TH1</t>
+  </si>
+  <si>
+    <t>PJDOM/PJ1</t>
+  </si>
+  <si>
+    <t>PJMX1/PJ2</t>
+  </si>
+  <si>
+    <t>PODOM/PO1</t>
+  </si>
+  <si>
+    <t>PRDOM/PR1</t>
+  </si>
+  <si>
+    <t>PRWMX/PRW</t>
+  </si>
+  <si>
+    <t>PRW</t>
+  </si>
+  <si>
+    <t>PWDOM/PW1</t>
+  </si>
+  <si>
+    <t>SBLOW/SB1</t>
+  </si>
+  <si>
+    <t>SPDOM/SP1</t>
+  </si>
+  <si>
+    <t>NER_LGFU</t>
+  </si>
+  <si>
+    <t>NWR_LGFU</t>
+  </si>
+  <si>
+    <t>lut_fu_sfu_lgfu_pft</t>
+  </si>
+  <si>
+    <t>The goal here is to rewrite the Caribou habitat onset age table with Provincial Standard Forest Unit instead of LGFU</t>
+  </si>
+  <si>
+    <t>PSFU</t>
+  </si>
+  <si>
+    <t>61-71</t>
+  </si>
+  <si>
+    <t>Merged BFDOM and CONMX</t>
+  </si>
+  <si>
+    <t>CLAYBELT</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>WINTER_USABLE</t>
+  </si>
+  <si>
+    <t>WINTER_PREFERRED</t>
+  </si>
+  <si>
+    <t>WINTER_SUITABLE</t>
+  </si>
+  <si>
+    <t>MATURE_CONIFER</t>
+  </si>
+  <si>
+    <t>CARIBOU_HABITAT</t>
+  </si>
+  <si>
+    <t>HABITAT_TYPE</t>
+  </si>
+  <si>
+    <t>SBDOM, SBMX1, SP1</t>
+  </si>
+  <si>
+    <t>Merged SBLOW, SP1 and SBMX1 - they are the same in terms of caribou habitat</t>
+  </si>
+  <si>
+    <t>PJMX1, PJ2</t>
+  </si>
+  <si>
+    <t>Merged PJMX1 and PJ2 - the same habitat</t>
+  </si>
+  <si>
+    <t>Merged OCLOW and LC1 - the same habitat</t>
+  </si>
+  <si>
+    <t>Merged PJDOM and PJ1 - the same habitat</t>
+  </si>
+  <si>
+    <t>PJDOM, PJ1</t>
+  </si>
+  <si>
+    <t>OCLOW, LC1</t>
+  </si>
+  <si>
+    <t>merged SBLOW, SB1 and SBOG - they are the same in terms of caribou habitat</t>
+  </si>
+  <si>
+    <t>SB1, SBOG, SBLOW</t>
+  </si>
+  <si>
+    <t>The goal here is to assign each provincial SFU with caribou habitat type.</t>
+  </si>
+  <si>
+    <t>SB1, SP1</t>
+  </si>
+  <si>
+    <t>This is the only one that I am not 100% comfortable with</t>
+  </si>
+  <si>
+    <t>WINTER1</t>
+  </si>
+  <si>
+    <t>WINTER2</t>
+  </si>
+  <si>
+    <t>Not Clay Belt</t>
+  </si>
+  <si>
+    <t>Clay Belt</t>
+  </si>
+  <si>
+    <t>`</t>
+  </si>
+  <si>
+    <t>LGFU</t>
+  </si>
+  <si>
+    <t>useable, preferred, refuge</t>
+  </si>
+  <si>
+    <t>useable and, refuge</t>
+  </si>
+  <si>
+    <t>This is good to use!</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -278,13 +527,28 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Courier New"/>
+      <family val="3"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -297,8 +561,62 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1" tint="0.34998626667073579"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -349,11 +667,63 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -367,7 +737,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
@@ -375,6 +744,36 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -396,23 +795,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>295275</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>154938</xdr:rowOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>352425</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>22</xdr:col>
-      <xdr:colOff>55622</xdr:colOff>
-      <xdr:row>30</xdr:row>
-      <xdr:rowOff>65839</xdr:rowOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>152400</xdr:colOff>
+      <xdr:row>45</xdr:row>
+      <xdr:rowOff>103760</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
+        <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{35607188-B572-ABD7-4C58-3F4C591C84DE}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FED12837-8E90-BFEB-C84E-6FBD01578D4B}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -428,8 +827,145 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6400800" y="154938"/>
-          <a:ext cx="11342747" cy="6197401"/>
+          <a:off x="5848350" y="285750"/>
+          <a:ext cx="7115175" cy="8962010"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>390526</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>127594</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>323850</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>162739</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6D94DE4E-B7E6-D81F-CC8F-044DDF0CA2E2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="13201651" y="1461094"/>
+          <a:ext cx="6638924" cy="5559645"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>390526</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>70312</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{12B19C7E-CFDF-438E-8537-C19DAD526FDE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8315326" y="57150"/>
+          <a:ext cx="6994986" cy="8810625"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>28576</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>3769</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>343047</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{752E43DD-A6A9-4208-8A35-B12B0C81FFAE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="14658976" y="1718269"/>
+          <a:ext cx="6410471" cy="5368331"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -448,9 +984,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -488,7 +1024,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -594,7 +1130,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -736,7 +1272,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -746,6 +1282,33 @@
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <threadedComment ref="B1" dT="2024-12-31T15:16:17.19" personId="{DD1F84D2-F0F8-48F7-BC38-1DFD7CC497C8}" id="{2A2B33F3-E54A-43C7-9B24-F9761397EC4D}">
     <text>From Larry's PIAM 2024</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
+<file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="A3" dT="2026-06-09T19:40:08.08" personId="{DD1F84D2-F0F8-48F7-BC38-1DFD7CC497C8}" id="{2962486B-8D99-4130-8A33-5C0AE0A274D5}">
+    <text>There is a look-up table available to map thousands of plan forest unit to provincial standard forest units. Most CM1.3 data will be mapped to PSFU then mapped to LGFU to determine caribou habitat</text>
+  </threadedComment>
+  <threadedComment ref="C3" dT="2024-12-31T15:16:17.19" personId="{DD1F84D2-F0F8-48F7-BC38-1DFD7CC497C8}" id="{7C908EB8-4275-4D83-8DF4-FB495EEC1BDF}">
+    <text>From Larry's PIAM 2024</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
+<file path=xl/threadedComments/threadedComment3.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="A13" dT="2026-06-09T20:15:47.81" personId="{DD1F84D2-F0F8-48F7-BC38-1DFD7CC497C8}" id="{4401C003-C0F5-4F5E-B99D-BFAE1416E019}">
+    <text>It should’ve been SBLOW/SB1, but in this context, it seems more appropriate to assign this to SPDOM/SP1</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
+<file path=xl/threadedComments/threadedComment4.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="A12" dT="2026-06-09T20:15:47.81" personId="{DD1F84D2-F0F8-48F7-BC38-1DFD7CC497C8}" id="{CEE603A1-4FDB-4D6E-91BE-F9B21160272F}">
+    <text>It should’ve been SBLOW/SB1, but in this context, it seems more appropriate to assign this to SPDOM/SP1</text>
   </threadedComment>
 </ThreadedComments>
 </file>
@@ -866,7 +1429,7 @@
   <dimension ref="A1:I52"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="1" max="1" width="10.42578125" customWidth="1"/>
     <col min="4" max="4" width="15.7109375" customWidth="1"/>
     <col min="5" max="5" width="15" customWidth="1"/>
     <col min="6" max="6" width="10.28515625" customWidth="1"/>
@@ -922,11 +1485,11 @@
       <c r="I2" s="6"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8" t="s">
+      <c r="B3" s="7"/>
+      <c r="C3" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D3" s="5"/>
@@ -956,13 +1519,13 @@
       <c r="I4" s="6"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D5" s="5"/>
@@ -973,13 +1536,13 @@
       <c r="I5" s="6"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D6" s="5"/>
@@ -993,7 +1556,7 @@
       <c r="A7" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="5" t="s">
         <v>5</v>
       </c>
       <c r="C7" s="5" t="s">
@@ -1011,13 +1574,13 @@
       <c r="I7" s="6"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D8" s="5"/>
@@ -1074,36 +1637,36 @@
       <c r="I10" s="6"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
-      <c r="H11" s="8"/>
-      <c r="I11" s="9"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="7"/>
+      <c r="I11" s="8"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="8" t="s">
+      <c r="A12" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="8"/>
-      <c r="C12" s="8" t="s">
+      <c r="B12" s="7"/>
+      <c r="C12" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="8"/>
-      <c r="G12" s="8"/>
-      <c r="H12" s="8"/>
-      <c r="I12" s="9"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="7"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="8"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
@@ -1150,51 +1713,51 @@
       <c r="I14" s="6"/>
     </row>
     <row r="15" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="13" t="s">
+      <c r="A15" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="13" t="s">
+      <c r="B15" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="C15" s="13" t="s">
+      <c r="C15" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="D15" s="13">
+      <c r="D15" s="12">
         <v>61</v>
       </c>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13">
+      <c r="E15" s="12"/>
+      <c r="F15" s="12">
         <v>41</v>
       </c>
-      <c r="G15" s="13"/>
-      <c r="H15" s="13"/>
-      <c r="I15" s="14"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="12"/>
+      <c r="I15" s="13"/>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="10" t="s">
+      <c r="A16" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="C16" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11"/>
-      <c r="G16" s="11"/>
-      <c r="H16" s="11"/>
-      <c r="I16" s="12"/>
+      <c r="C16" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="10"/>
+      <c r="H16" s="10"/>
+      <c r="I16" s="11"/>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="8" t="s">
+      <c r="A17" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="C17" s="7" t="s">
         <v>38</v>
       </c>
       <c r="D17" s="5"/>
@@ -1205,13 +1768,13 @@
       <c r="I17" s="6"/>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="8" t="s">
+      <c r="A18" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B18" s="8" t="s">
+      <c r="B18" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C18" s="8" t="s">
+      <c r="C18" s="7" t="s">
         <v>38</v>
       </c>
       <c r="D18" s="5"/>
@@ -1222,13 +1785,13 @@
       <c r="I18" s="6"/>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="8" t="s">
+      <c r="A19" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="B19" s="8" t="s">
+      <c r="B19" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="C19" s="7" t="s">
         <v>38</v>
       </c>
       <c r="D19" s="5"/>
@@ -1359,13 +1922,13 @@
       <c r="I25" s="6"/>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" s="8" t="s">
+      <c r="A26" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B26" s="8" t="s">
+      <c r="B26" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="C26" s="7" t="s">
         <v>38</v>
       </c>
       <c r="D26" s="5"/>
@@ -1376,13 +1939,13 @@
       <c r="I26" s="6"/>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="8" t="s">
+      <c r="A27" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B27" s="8" t="s">
+      <c r="B27" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="C27" s="8" t="s">
+      <c r="C27" s="7" t="s">
         <v>38</v>
       </c>
       <c r="D27" s="5"/>
@@ -1393,13 +1956,13 @@
       <c r="I27" s="6"/>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" s="8" t="s">
+      <c r="A28" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B28" s="8" t="s">
+      <c r="B28" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C28" s="8" t="s">
+      <c r="C28" s="7" t="s">
         <v>38</v>
       </c>
       <c r="D28" s="5"/>
@@ -1410,13 +1973,13 @@
       <c r="I28" s="6"/>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" s="8" t="s">
+      <c r="A29" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="B29" s="8" t="s">
+      <c r="B29" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="C29" s="8" t="s">
+      <c r="C29" s="7" t="s">
         <v>38</v>
       </c>
       <c r="D29" s="5"/>
@@ -1427,13 +1990,13 @@
       <c r="I29" s="6"/>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" s="8" t="s">
+      <c r="A30" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="B30" s="8" t="s">
+      <c r="B30" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="C30" s="8" t="s">
+      <c r="C30" s="7" t="s">
         <v>38</v>
       </c>
       <c r="D30" s="5"/>
@@ -1463,25 +2026,25 @@
       <c r="I31" s="6"/>
     </row>
     <row r="32" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="13" t="s">
+      <c r="A32" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="B32" s="13" t="s">
+      <c r="B32" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="C32" s="13" t="s">
-        <v>38</v>
-      </c>
-      <c r="D32" s="13"/>
-      <c r="E32" s="13"/>
-      <c r="F32" s="13"/>
-      <c r="G32" s="13" t="s">
+      <c r="C32" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="D32" s="12"/>
+      <c r="E32" s="12"/>
+      <c r="F32" s="12"/>
+      <c r="G32" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="H32" s="13" t="s">
+      <c r="H32" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="I32" s="14"/>
+      <c r="I32" s="13"/>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
@@ -1571,6 +2134,2015 @@
     <row r="52" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B52" t="s">
         <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1659DA6-F213-4B38-8E83-FD2DB6EB297E}">
+  <dimension ref="A1:I74"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.42578125" customWidth="1"/>
+    <col min="2" max="2" width="18.5703125" customWidth="1"/>
+    <col min="3" max="3" width="15.42578125" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" customWidth="1"/>
+    <col min="6" max="6" width="15" customWidth="1"/>
+    <col min="7" max="7" width="10.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="22" t="s">
+        <v>72</v>
+      </c>
+      <c r="B4" s="22" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="22" t="s">
+        <v>47</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5">
+        <v>61</v>
+      </c>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="7"/>
+      <c r="B5" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5"/>
+      <c r="I5" s="5"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="22" t="s">
+        <v>72</v>
+      </c>
+      <c r="B6" s="22" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6" s="22" t="s">
+        <v>2</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5">
+        <v>71</v>
+      </c>
+      <c r="H6" s="5"/>
+      <c r="I6" s="5"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5">
+        <v>71</v>
+      </c>
+      <c r="H7" s="5"/>
+      <c r="I7" s="5"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="7"/>
+      <c r="B8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
+      <c r="I8" s="5"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="7"/>
+      <c r="B9" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="5"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="29" t="s">
+        <v>79</v>
+      </c>
+      <c r="B10" s="29" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" s="29" t="s">
+        <v>5</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E10" s="5">
+        <v>51</v>
+      </c>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="7"/>
+      <c r="B11" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
+      <c r="I11" s="5"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="26" t="s">
+        <v>82</v>
+      </c>
+      <c r="B12" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E12" s="5">
+        <v>41</v>
+      </c>
+      <c r="F12" s="5">
+        <v>61</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="H12" s="5"/>
+      <c r="I12" s="5"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E13" s="5">
+        <v>41</v>
+      </c>
+      <c r="F13" s="5">
+        <v>61</v>
+      </c>
+      <c r="G13" s="5">
+        <v>41</v>
+      </c>
+      <c r="H13" s="5"/>
+      <c r="I13" s="5"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="7"/>
+      <c r="B14" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="7"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="7"/>
+      <c r="B15" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C15" s="7"/>
+      <c r="D15" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="7"/>
+      <c r="I15" s="7"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="B16" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="C16" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E16" s="5">
+        <v>61</v>
+      </c>
+      <c r="F16" s="5"/>
+      <c r="G16" s="5">
+        <v>41</v>
+      </c>
+      <c r="H16" s="5"/>
+      <c r="I16" s="5"/>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" s="27" t="s">
+        <v>89</v>
+      </c>
+      <c r="B17" s="27" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" s="27" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E17" s="5">
+        <v>41</v>
+      </c>
+      <c r="F17" s="5">
+        <v>101</v>
+      </c>
+      <c r="G17" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="H17" s="5"/>
+      <c r="I17" s="5"/>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="B18" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="E18" s="14">
+        <v>61</v>
+      </c>
+      <c r="F18" s="14"/>
+      <c r="G18" s="14">
+        <v>41</v>
+      </c>
+      <c r="H18" s="14"/>
+      <c r="I18" s="14"/>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" s="7"/>
+      <c r="B19" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C19" s="7"/>
+      <c r="D19" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="E19" s="14"/>
+      <c r="F19" s="14"/>
+      <c r="G19" s="14"/>
+      <c r="H19" s="14"/>
+      <c r="I19" s="14"/>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" s="7"/>
+      <c r="B20" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C20" s="7"/>
+      <c r="D20" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="E20" s="14"/>
+      <c r="F20" s="14"/>
+      <c r="G20" s="14"/>
+      <c r="H20" s="14"/>
+      <c r="I20" s="14"/>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="7"/>
+      <c r="B21" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C21" s="7"/>
+      <c r="D21" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="E21" s="14"/>
+      <c r="F21" s="14"/>
+      <c r="G21" s="14"/>
+      <c r="H21" s="14"/>
+      <c r="I21" s="14"/>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" s="7"/>
+      <c r="B22" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C22" s="7"/>
+      <c r="D22" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="E22" s="14"/>
+      <c r="F22" s="14"/>
+      <c r="G22" s="14"/>
+      <c r="H22" s="14"/>
+      <c r="I22" s="14"/>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" s="28" t="s">
+        <v>79</v>
+      </c>
+      <c r="B23" s="28" t="s">
+        <v>28</v>
+      </c>
+      <c r="C23" s="28"/>
+      <c r="D23" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="E23" s="14">
+        <v>51</v>
+      </c>
+      <c r="F23" s="14"/>
+      <c r="G23" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="H23" s="14"/>
+      <c r="I23" s="14"/>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="B24" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C24" s="14"/>
+      <c r="D24" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="E24" s="14">
+        <v>51</v>
+      </c>
+      <c r="F24" s="14"/>
+      <c r="G24" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="H24" s="14"/>
+      <c r="I24" s="14"/>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" s="7"/>
+      <c r="B25" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="C25" s="7"/>
+      <c r="D25" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="E25" s="14"/>
+      <c r="F25" s="14"/>
+      <c r="G25" s="14"/>
+      <c r="H25" s="14"/>
+      <c r="I25" s="14"/>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" s="25" t="s">
+        <v>82</v>
+      </c>
+      <c r="B26" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="C26" s="25"/>
+      <c r="D26" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="E26" s="14">
+        <v>41</v>
+      </c>
+      <c r="F26" s="14">
+        <v>61</v>
+      </c>
+      <c r="G26" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="H26" s="14"/>
+      <c r="I26" s="14"/>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27" s="15" t="s">
+        <v>83</v>
+      </c>
+      <c r="B27" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="C27" s="15"/>
+      <c r="D27" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="E27" s="14">
+        <v>41</v>
+      </c>
+      <c r="F27" s="14">
+        <v>61</v>
+      </c>
+      <c r="G27" s="14">
+        <v>41</v>
+      </c>
+      <c r="H27" s="14"/>
+      <c r="I27" s="14"/>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28" s="7"/>
+      <c r="B28" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C28" s="7"/>
+      <c r="D28" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="E28" s="14"/>
+      <c r="F28" s="14"/>
+      <c r="G28" s="14"/>
+      <c r="H28" s="14"/>
+      <c r="I28" s="14"/>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29" s="7"/>
+      <c r="B29" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="C29" s="7"/>
+      <c r="D29" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="E29" s="14"/>
+      <c r="F29" s="14"/>
+      <c r="G29" s="14"/>
+      <c r="H29" s="14"/>
+      <c r="I29" s="14"/>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="B30" s="21" t="s">
+        <v>30</v>
+      </c>
+      <c r="C30" s="21"/>
+      <c r="D30" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="E30" s="14">
+        <v>61</v>
+      </c>
+      <c r="F30" s="14"/>
+      <c r="G30" s="14">
+        <v>41</v>
+      </c>
+      <c r="H30" s="14"/>
+      <c r="I30" s="14"/>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31" s="23" t="s">
+        <v>89</v>
+      </c>
+      <c r="B31" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="C31" s="23"/>
+      <c r="D31" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="E31" s="14">
+        <v>41</v>
+      </c>
+      <c r="F31" s="14">
+        <v>101</v>
+      </c>
+      <c r="G31" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="H31" s="14"/>
+      <c r="I31" s="14"/>
+    </row>
+    <row r="32" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="B32" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="C32" s="24"/>
+      <c r="D32" s="32" t="s">
+        <v>38</v>
+      </c>
+      <c r="E32" s="12">
+        <v>41</v>
+      </c>
+      <c r="F32" s="12">
+        <v>101</v>
+      </c>
+      <c r="G32" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="H32" s="12"/>
+      <c r="I32" s="12"/>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33" s="9"/>
+      <c r="B33" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C33" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="D33" s="33" t="s">
+        <v>38</v>
+      </c>
+      <c r="E33" s="10"/>
+      <c r="F33" s="10"/>
+      <c r="G33" s="10"/>
+      <c r="H33" s="10"/>
+      <c r="I33" s="10"/>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34" s="7"/>
+      <c r="B34" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C34" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D34" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="E34" s="5"/>
+      <c r="F34" s="5"/>
+      <c r="G34" s="5"/>
+      <c r="H34" s="5"/>
+      <c r="I34" s="5"/>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35" s="7"/>
+      <c r="B35" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C35" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D35" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="E35" s="5"/>
+      <c r="F35" s="5"/>
+      <c r="G35" s="5"/>
+      <c r="H35" s="5"/>
+      <c r="I35" s="5"/>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36" s="7"/>
+      <c r="B36" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C36" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D36" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="E36" s="5"/>
+      <c r="F36" s="5"/>
+      <c r="G36" s="5"/>
+      <c r="H36" s="5"/>
+      <c r="I36" s="5"/>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A37" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C37" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="D37" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="E37" s="5"/>
+      <c r="F37" s="5"/>
+      <c r="G37" s="5"/>
+      <c r="H37" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="I37" s="5"/>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A38" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D38" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="E38" s="5"/>
+      <c r="F38" s="5"/>
+      <c r="G38" s="5"/>
+      <c r="H38" s="5">
+        <v>51</v>
+      </c>
+      <c r="I38" s="5">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A39" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D39" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="E39" s="5"/>
+      <c r="F39" s="5"/>
+      <c r="G39" s="5"/>
+      <c r="H39" s="5">
+        <v>41</v>
+      </c>
+      <c r="I39" s="5">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A40" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D40" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="E40" s="5"/>
+      <c r="F40" s="5"/>
+      <c r="G40" s="5"/>
+      <c r="H40" s="5">
+        <v>51</v>
+      </c>
+      <c r="I40" s="5"/>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A41" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B41" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D41" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="E41" s="5"/>
+      <c r="F41" s="5"/>
+      <c r="G41" s="5"/>
+      <c r="H41" s="5"/>
+      <c r="I41" s="5"/>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A42" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D42" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="E42" s="5"/>
+      <c r="F42" s="5"/>
+      <c r="G42" s="5"/>
+      <c r="H42" s="5">
+        <v>41</v>
+      </c>
+      <c r="I42" s="5">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A43" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D43" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="E43" s="5"/>
+      <c r="F43" s="5"/>
+      <c r="G43" s="5"/>
+      <c r="H43" s="5">
+        <v>51</v>
+      </c>
+      <c r="I43" s="5"/>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A44" s="7"/>
+      <c r="B44" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C44" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D44" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="E44" s="5"/>
+      <c r="F44" s="5"/>
+      <c r="G44" s="5"/>
+      <c r="H44" s="5"/>
+      <c r="I44" s="5"/>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A45" s="7"/>
+      <c r="B45" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C45" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="D45" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="E45" s="5"/>
+      <c r="F45" s="5"/>
+      <c r="G45" s="5"/>
+      <c r="H45" s="5"/>
+      <c r="I45" s="5"/>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A46" s="7"/>
+      <c r="B46" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C46" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="D46" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="E46" s="5"/>
+      <c r="F46" s="5"/>
+      <c r="G46" s="5"/>
+      <c r="H46" s="5"/>
+      <c r="I46" s="5"/>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A47" s="7"/>
+      <c r="B47" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C47" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="D47" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="E47" s="5"/>
+      <c r="F47" s="5"/>
+      <c r="G47" s="5"/>
+      <c r="H47" s="5"/>
+      <c r="I47" s="5"/>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A48" s="7"/>
+      <c r="B48" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C48" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="D48" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="E48" s="5"/>
+      <c r="F48" s="5"/>
+      <c r="G48" s="5"/>
+      <c r="H48" s="5"/>
+      <c r="I48" s="5"/>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A49" s="5"/>
+      <c r="B49" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C49" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D49" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="E49" s="5"/>
+      <c r="F49" s="5"/>
+      <c r="G49" s="5"/>
+      <c r="H49" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="I49" s="5"/>
+    </row>
+    <row r="50" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="12"/>
+      <c r="B50" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C50" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="D50" s="32" t="s">
+        <v>38</v>
+      </c>
+      <c r="E50" s="12"/>
+      <c r="F50" s="12"/>
+      <c r="G50" s="12"/>
+      <c r="H50" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="I50" s="12" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A54" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="B54" s="18"/>
+      <c r="C54" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="D54" s="18" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A55" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="B55" s="17"/>
+      <c r="C55" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="D55" s="17" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A56" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="B56" s="16"/>
+      <c r="C56" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="D56" s="16" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A57" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="B57" s="16"/>
+      <c r="C57" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="D57" s="16" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A58" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="B58" s="16"/>
+      <c r="C58" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="D58" s="16" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A59" s="16" t="s">
+        <v>73</v>
+      </c>
+      <c r="B59" s="16"/>
+      <c r="C59" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D59" s="16" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A60" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="B60" s="16"/>
+      <c r="C60" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="D60" s="16" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A61" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="B61" s="16"/>
+      <c r="C61" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="D61" s="16" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A62" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="B62" s="16"/>
+      <c r="C62" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="D62" s="16" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A63" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="B63" s="16"/>
+      <c r="C63" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="D63" s="16" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A64" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="B64" s="16"/>
+      <c r="C64" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="D64" s="16" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A65" s="16" t="s">
+        <v>80</v>
+      </c>
+      <c r="B65" s="16"/>
+      <c r="C65" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="D65" s="16" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A66" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="B66" s="16"/>
+      <c r="C66" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="D66" s="16" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A67" s="16" t="s">
+        <v>82</v>
+      </c>
+      <c r="B67" s="16"/>
+      <c r="C67" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="D67" s="16" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68" s="16" t="s">
+        <v>83</v>
+      </c>
+      <c r="B68" s="16"/>
+      <c r="C68" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="D68" s="16" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A69" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="B69" s="16"/>
+      <c r="C69" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="D69" s="16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="B70" s="16"/>
+      <c r="C70" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="D70" s="16" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A71" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="B71" s="16"/>
+      <c r="C71" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="D71" s="16" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72" s="16" t="s">
+        <v>88</v>
+      </c>
+      <c r="B72" s="16"/>
+      <c r="C72" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="D72" s="16" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="B73" s="16"/>
+      <c r="C73" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="D73" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A74" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="B74" s="16"/>
+      <c r="C74" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="D74" s="16" t="s">
+        <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5EABE0A-1E91-4AE5-B50B-40D8BEE1B97E}">
+  <dimension ref="A1:L23"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="4" max="4" width="13.85546875" customWidth="1"/>
+    <col min="5" max="5" width="17" customWidth="1"/>
+    <col min="6" max="6" width="15.28515625" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" customWidth="1"/>
+    <col min="8" max="8" width="17.5703125" customWidth="1"/>
+    <col min="9" max="10" width="18" customWidth="1"/>
+    <col min="11" max="11" width="19.5703125" customWidth="1"/>
+    <col min="12" max="12" width="19.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="B3" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="E3" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="F3" s="18" t="s">
+        <v>101</v>
+      </c>
+      <c r="G3" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="H3" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="I3" s="18" t="s">
+        <v>103</v>
+      </c>
+      <c r="J3" s="18" t="s">
+        <v>104</v>
+      </c>
+      <c r="K3" s="18" t="s">
+        <v>105</v>
+      </c>
+      <c r="L3" s="19" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="L4" s="6" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5">
+        <v>71</v>
+      </c>
+      <c r="H5" s="5"/>
+      <c r="I5" s="5"/>
+      <c r="J5" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="L5" s="6"/>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="E6" s="5">
+        <v>51</v>
+      </c>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="H6" s="5"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="L6" s="6" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="E7" s="5">
+        <v>41</v>
+      </c>
+      <c r="F7" s="5">
+        <v>61</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="H7" s="5"/>
+      <c r="I7" s="5"/>
+      <c r="J7" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="L7" s="6" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="E8" s="5">
+        <v>41</v>
+      </c>
+      <c r="F8" s="5">
+        <v>61</v>
+      </c>
+      <c r="G8" s="5">
+        <v>41</v>
+      </c>
+      <c r="H8" s="5"/>
+      <c r="I8" s="5"/>
+      <c r="J8" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="L8" s="6" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="E9" s="5">
+        <v>61</v>
+      </c>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5">
+        <v>41</v>
+      </c>
+      <c r="H9" s="5"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="L9" s="6" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="E10" s="14">
+        <v>51</v>
+      </c>
+      <c r="F10" s="14"/>
+      <c r="G10" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="H10" s="14"/>
+      <c r="I10" s="14"/>
+      <c r="J10" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="L10" s="15"/>
+    </row>
+    <row r="11" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="E11" s="12">
+        <v>41</v>
+      </c>
+      <c r="F11" s="12">
+        <v>101</v>
+      </c>
+      <c r="G11" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="H11" s="12"/>
+      <c r="I11" s="12"/>
+      <c r="J11" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="K11" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="L11" s="13" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="I12" s="5"/>
+      <c r="J12" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="K12" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="L12" s="6"/>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="5">
+        <v>51</v>
+      </c>
+      <c r="I13" s="5">
+        <v>101</v>
+      </c>
+      <c r="J13" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="K13" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="L13" s="6" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="5">
+        <v>41</v>
+      </c>
+      <c r="I14" s="5">
+        <v>71</v>
+      </c>
+      <c r="J14" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="K14" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="L14" s="6"/>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="E15" s="5"/>
+      <c r="F15" s="5"/>
+      <c r="G15" s="5"/>
+      <c r="H15" s="5">
+        <v>51</v>
+      </c>
+      <c r="I15" s="5"/>
+      <c r="J15" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="K15" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="L15" s="6"/>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A16" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="E16" s="5"/>
+      <c r="F16" s="5"/>
+      <c r="G16" s="5"/>
+      <c r="H16" s="5">
+        <v>51</v>
+      </c>
+      <c r="I16" s="5"/>
+      <c r="J16" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="K16" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="L16" s="6"/>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A17" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
+      <c r="G17" s="5"/>
+      <c r="H17" s="5">
+        <v>41</v>
+      </c>
+      <c r="I17" s="5">
+        <v>71</v>
+      </c>
+      <c r="J17" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="K17" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="L17" s="6"/>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H23" t="s">
+        <v>123</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D76CE8B1-9850-4A90-9F28-0273EC006EA2}">
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.7109375" customWidth="1"/>
+    <col min="2" max="2" width="20.140625" customWidth="1"/>
+    <col min="3" max="3" width="14.140625" customWidth="1"/>
+    <col min="4" max="4" width="18.140625" customWidth="1"/>
+    <col min="5" max="5" width="14" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="35" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="B2" s="18" t="s">
+        <v>124</v>
+      </c>
+      <c r="C2" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="D2" s="18" t="s">
+        <v>104</v>
+      </c>
+      <c r="E2" s="18" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="38" t="s">
+        <v>82</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="F6" s="34" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="38" t="s">
+        <v>83</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="36" t="s">
+        <v>90</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="F8" s="34" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="37" t="s">
+        <v>52</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="39" t="s">
+        <v>89</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="36" t="s">
+        <v>89</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="38" t="s">
+        <v>90</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="38" t="s">
+        <v>82</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="36" t="s">
+        <v>52</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="38" t="s">
+        <v>83</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>120</v>
       </c>
     </row>
   </sheetData>

</xml_diff>